<commit_message>
feat: Implement Excel document generation for research projects
- Added decision document 0007 for Excel document generation strategy using ClosedXML.Report with embedded templates.
- Created ProyectosReport class to handle multi-sheet Excel reports for various project types.
- Updated Dependency Injection to register ProyectosReport.
- Implemented frontend functionality to generate and download the "Anexo 4" Excel report for projects.
- Modified existing templates and added new ones for project types.
- Adjusted endpoint authorization to include role checks for document generation.
</commit_message>
<xml_diff>
--- a/Dashboard_v2/src/Infrastructure/Templates/AnexoProyectos.xlsx
+++ b/Dashboard_v2/src/Infrastructure/Templates/AnexoProyectos.xlsx
@@ -97,6 +97,66 @@
     <x:t>Publicaciones derivadas del proyecto (DOI / URL)</x:t>
   </x:si>
   <x:si>
+    <x:t>{{item.CodigoProyecto}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.TituloProyecto}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.NombrePrograma}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.JefeProyecto}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.CorreoJefeProyecto}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.TotalMiembros}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.MiembrosUH}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.Estudiantes}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.EstudiantesContratados}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.Clasificacion}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.TributaFormacionDoctoral}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.TributaDesarrolloLocal}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.ContribucionSectoresEstrategicos}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.ContribucionEjesEstrategicos}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.FechaInicio}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.FechaCierre}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.EntidadEjecutoraPrincipal}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.EntidadEjecutoraParticipante}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.EstadoEjecucion}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.PublicacionesDerivadas}}</x:t>
+  </x:si>
+  <x:si>
     <x:t/>
   </x:si>
   <x:si>
@@ -112,18 +172,27 @@
     <x:t>Empresa</x:t>
   </x:si>
   <x:si>
+    <x:t>{{item.Empresa}}</x:t>
+  </x:si>
+  <x:si>
     <x:t>Proyectos PNE</x:t>
   </x:si>
   <x:si>
     <x:t>Entidad no empresarial con la que se desarrolla el proyecto</x:t>
   </x:si>
   <x:si>
+    <x:t>{{item.EntidadNoEmpresarial}}</x:t>
+  </x:si>
+  <x:si>
     <x:t>Proyectos PDL</x:t>
   </x:si>
   <x:si>
     <x:t>Municipio</x:t>
   </x:si>
   <x:si>
+    <x:t>{{item.Municipio}}</x:t>
+  </x:si>
+  <x:si>
     <x:t>Proyectos PRCI</x:t>
   </x:si>
   <x:si>
@@ -133,12 +202,21 @@
     <x:t>Con Términos de referencia</x:t>
   </x:si>
   <x:si>
+    <x:t>{{item.FuenteFinanciacion}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.ConTerminosReferencia}}</x:t>
+  </x:si>
+  <x:si>
     <x:t>Proyectos PNAP</x:t>
   </x:si>
   <x:si>
     <x:t>Financiamiento UH</x:t>
   </x:si>
   <x:si>
+    <x:t>{{item.FinanciamientoUH}}</x:t>
+  </x:si>
+  <x:si>
     <x:t>Nuevas Aplicaciones</x:t>
   </x:si>
   <x:si>
@@ -146,6 +224,12 @@
   </x:si>
   <x:si>
     <x:t>Situación (aprobado e inicia este año, pendiente de aprobación, rechazado)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.TipoProyecto}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{item.Situacion}}</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -262,7 +346,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellXfs>
@@ -638,66 +722,66 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:20">
       <x:c r="A6" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -725,7 +809,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:20">
       <x:c r="A1" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:20" ht="50" customHeight="1">
@@ -795,66 +879,66 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:20">
       <x:c r="A6" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -882,7 +966,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:20">
       <x:c r="A1" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:20" ht="50" customHeight="1">
@@ -952,66 +1036,66 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:20">
       <x:c r="A6" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1039,7 +1123,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:20">
       <x:c r="A1" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:20" ht="50" customHeight="1">
@@ -1050,7 +1134,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D4" s="2" t="s">
         <x:v>4</x:v>
@@ -1109,66 +1193,66 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:20">
       <x:c r="A6" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1196,7 +1280,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:20">
       <x:c r="A1" s="1" t="s">
-        <x:v>26</x:v>
+        <x:v>47</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:20" ht="50" customHeight="1">
@@ -1207,7 +1291,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D4" s="2" t="s">
         <x:v>4</x:v>
@@ -1266,66 +1350,66 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:20">
       <x:c r="A6" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1353,7 +1437,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:20">
       <x:c r="A1" s="1" t="s">
-        <x:v>28</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:20" ht="50" customHeight="1">
@@ -1364,7 +1448,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="2" t="s">
-        <x:v>29</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D4" s="2" t="s">
         <x:v>4</x:v>
@@ -1423,66 +1507,66 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:20">
       <x:c r="A6" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1510,7 +1594,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:21">
       <x:c r="A1" s="1" t="s">
-        <x:v>30</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:21" ht="50" customHeight="1">
@@ -1521,7 +1605,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D4" s="2" t="s">
         <x:v>4</x:v>
@@ -1551,7 +1635,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="M4" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="N4" s="2" t="s">
         <x:v>13</x:v>
@@ -1583,69 +1667,69 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="K5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="U5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:21">
       <x:c r="A6" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1673,7 +1757,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:20">
       <x:c r="A1" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>58</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:20" ht="50" customHeight="1">
@@ -1711,7 +1795,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="L4" s="2" t="s">
-        <x:v>34</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="M4" s="2" t="s">
         <x:v>13</x:v>
@@ -1743,66 +1827,66 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="K5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:20">
       <x:c r="A6" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1830,7 +1914,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:11">
       <x:c r="A1" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:11" ht="50" customHeight="1">
@@ -1844,7 +1928,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D4" s="2" t="s">
-        <x:v>36</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="E4" s="2" t="s">
         <x:v>6</x:v>
@@ -1865,47 +1949,47 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="K4" s="2" t="s">
-        <x:v>37</x:v>
+        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:11">
       <x:c r="A5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="K5" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:11">
       <x:c r="A6" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>